<commit_message>
chore: add numberUtils test
</commit_message>
<xml_diff>
--- a/test/Stock Summary-12345678.xlsx
+++ b/test/Stock Summary-12345678.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/k/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/k/work/KAnggara75/IDXStock/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BA1B79-0600-9D4C-9E87-F971A508AA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB8C603-DD1D-6244-B78A-9352E1B0D9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="40960" windowHeight="25600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>